<commit_message>
git add . git commit git push
</commit_message>
<xml_diff>
--- a/data/budget_fil.xlsx
+++ b/data/budget_fil.xlsx
@@ -509,45 +509,19 @@
           <t>Mad</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="D2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="E2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="F2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="G2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="H2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="I2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="J2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="K2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="L2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="M2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="N2" t="n">
-        <v>5000</v>
-      </c>
-      <c r="O2" t="n">
-        <v>60000</v>
-      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr"/>
+      <c r="O2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -558,45 +532,19 @@
           <t>Boliglån</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E3" t="n">
-        <v>7000</v>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>7000</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>7000</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="n">
-        <v>7000</v>
-      </c>
-      <c r="O3" t="n">
-        <v>28000</v>
-      </c>
+      <c r="C3" t="inlineStr"/>
+      <c r="D3" t="inlineStr"/>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr"/>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr"/>
+      <c r="O3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">

</xml_diff>